<commit_message>
DATATABLE 수정_ 1번방 LOCKER 연결
</commit_message>
<xml_diff>
--- a/EXCEL/SILENT_Asset_Datatable.xlsx
+++ b/EXCEL/SILENT_Asset_Datatable.xlsx
@@ -1138,7 +1138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F92"/>
+  <dimension ref="A1:F95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="10" customWidth="1" style="10" min="1" max="1"/>
@@ -1357,17 +1357,17 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>4칸 다이얼 자물쇠</t>
+          <t>2번 방 4칸 다이얼 자물쇠 (Lock_02 모델)</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Prefabs/Common/DialLock_4</t>
+          <t>Assets/2.Model/Prefabs/R02/R02_Lock</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Shared</t>
+          <t>Room2</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
@@ -1387,17 +1387,17 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>5칸 다이얼 자물쇠</t>
+          <t>4번 방 5칸 다이얼 자물쇠 (Padlock_5Dial_1to9 모델)</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Prefabs/Common/DialLock_5</t>
+          <t>Assets/2.Model/Prefabs/R04/R04_Lock</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Shared</t>
+          <t>Room4</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -1417,17 +1417,17 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>6칸 색 다이얼 자물쇠</t>
+          <t>7번 방 A 6칸 색 다이얼 자물쇠 (안내 글자 LISTEN)</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Prefabs/Common/DialLock_6</t>
+          <t>Assets/2.Model/Prefabs/R07/R07_Lock</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Shared</t>
+          <t>Room7</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -1443,70 +1443,68 @@
     </row>
     <row r="14">
       <c r="A14" s="8" t="n">
-        <v>13008</v>
+        <v>13010</v>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>글자 표시판</t>
+          <t>액자</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Prefabs/Common/LetterSign</t>
+          <t>Prefabs/R2/Frame_100x80</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Shared</t>
+          <t>Room2</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>CMN-05</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="n">
-        <v>14006</v>
-      </c>
+          <t>R2B-01</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="n">
-        <v>13010</v>
+        <v>13011</v>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>액자</t>
+          <t>단서 화살표</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Prefabs/R2/Frame_100x80</t>
+          <t>Prefabs/R3/Arrow_Painted</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Room2</t>
+          <t>Room3</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>R2B-01</t>
+          <t>R3A-01</t>
         </is>
       </c>
       <c r="F15" s="8" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n">
-        <v>13011</v>
+        <v>13012</v>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>단서 화살표</t>
+          <t>3번 방 화살표 콘솔</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Prefabs/R3/Arrow_Painted</t>
+          <t>Assets/2.Model/Prefabs/R03/R03_ArrowConsole</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
@@ -1516,83 +1514,87 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>R3A-01</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="n"/>
+          <t>R3B-01</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>14001|14002|14004|14007</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n">
-        <v>13012</v>
+        <v>13013</v>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>화살표 콘솔</t>
+          <t>4번 방 배선 콘솔 (뚜껑 열린 모델 4_Lock_Opened)</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Prefabs/R3/ArrowConsole</t>
+          <t>Assets/2.Model/Prefabs/R04/R04_CableConsole</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>Room3</t>
+          <t>Room4</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>R3B-01</t>
+          <t>R4B-01</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>14001|14002|14004|14007</t>
+          <t>14001|14002</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n">
-        <v>13013</v>
+        <v>13014</v>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>배선 콘솔</t>
+          <t>공식판</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>Prefabs/R4/WireConsole</t>
+          <t>Prefabs/R5/FormulaBoard</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>Room4</t>
+          <t>Room5</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>R4B-01</t>
+          <t>R5A-01</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>14001|14002</t>
+          <t>14007</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="n">
-        <v>13014</v>
+        <v>13016</v>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>공식판</t>
+          <t>종이</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Prefabs/R5/FormulaBoard</t>
+          <t>Prefabs/R5/TrianglePaper</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
@@ -1602,7 +1604,7 @@
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>R5A-01</t>
+          <t>R5A-02</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -1613,46 +1615,44 @@
     </row>
     <row r="20">
       <c r="A20" s="8" t="n">
-        <v>13016</v>
+        <v>13017</v>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>종이</t>
+          <t>켜진 TV</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Prefabs/R5/TrianglePaper</t>
+          <t>Prefabs/R6/TV_142x80</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>Room5</t>
+          <t>Room6</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>R5A-02</t>
-        </is>
-      </c>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>14007</t>
-        </is>
+          <t>R6B-01</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="n">
+        <v>14007</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="n">
-        <v>13017</v>
+        <v>13018</v>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>켜진 TV</t>
+          <t>꺼진 TV (방 프리팹에 직접 배치, 앵커 없음)</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>Prefabs/R6/TV_142x80</t>
+          <t>Prefabs/R6/TV_Off</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
@@ -1662,77 +1662,75 @@
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>R6B-01</t>
-        </is>
-      </c>
-      <c r="F21" s="8" t="n">
-        <v>14007</v>
-      </c>
+          <t>R6B-02</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="8" t="n">
-        <v>13018</v>
+        <v>13019</v>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>꺼진 TV (방 프리팹에 직접 배치, 앵커 없음)</t>
+          <t>배선 콘솔 받침대</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>Prefabs/R6/TV_Off</t>
+          <t>Prefabs/R4/WireConsole_Stand</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>Room6</t>
+          <t>Room4</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>R6B-02</t>
+          <t>R4B-01</t>
         </is>
       </c>
       <c r="F22" s="8" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="8" t="n">
-        <v>13019</v>
+        <v>13020</v>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>배선 콘솔 받침대</t>
+          <t>A 1번 방 기본 프리팹 (A·B 공통: 맵 R01_Structure + 천장 Ceiling.007 + 문 막기 dver' + 앵커 R01_Points)</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Prefabs/R4/WireConsole_Stand</t>
+          <t>Assets/2.Model/Prefabs/R01/SILENT_Room_01_Final/Prefabs/Room_01_Final</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>Room4</t>
+          <t>RoomA</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>R4B-01</t>
+          <t>R1A-00</t>
         </is>
       </c>
       <c r="F23" s="8" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="8" t="n">
-        <v>13020</v>
+        <v>13021</v>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>A 1번 방 기본 프리팹 (A·B 공통: 맵 R01_Structure + 천장 Ceiling.007 + 문 막기 dver' + 앵커 R01_Points)</t>
+          <t>A 2번 방 프리팹 (천장 뺀 맵 R02_Structure + 앵커 R02_Points)</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R01/SILENT_Room_01_Final/Prefabs/Room_01_Final</t>
+          <t>Assets/2.Model/Prefabs/R02/SILENT_Room_02/Prefabs/SILENT_Room_02_Structure</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
@@ -1742,23 +1740,23 @@
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>R1A-00</t>
+          <t>R2A-00</t>
         </is>
       </c>
       <c r="F24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="8" t="n">
-        <v>13021</v>
+        <v>13022</v>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>A 2번 방 프리팹 (천장 뺀 맵 R02_Structure + 앵커 R02_Points)</t>
+          <t>A 3번 방 프리팹 (SILENT_Room_03_Structure, A·B 같은 방 껍데기)</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R02/SILENT_Room_02/Prefabs/SILENT_Room_02_Structure</t>
+          <t>Assets/2.Model/Prefabs/R03/SILENT_Room_03/Prefabs/SILENT_Room_03_Structure</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
@@ -1768,23 +1766,23 @@
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>R2A-00</t>
+          <t>R3A-00</t>
         </is>
       </c>
       <c r="F25" s="8" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="8" t="n">
-        <v>13022</v>
+        <v>13023</v>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>A 3번 방 프리팹 (SILENT_Room_03_Structure, A·B 같은 방 껍데기)</t>
+          <t>A 4번 방 프리팹 (SILENT_Room_04_Structure, A·B 같은 방 껍데기)</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R03/SILENT_Room_03/Prefabs/SILENT_Room_03_Structure</t>
+          <t>Assets/2.Model/Prefabs/R04/SILENT_Room_04/Prefabs/SILENT_Room_04_Structure</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
@@ -1794,23 +1792,23 @@
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>R3A-00</t>
+          <t>R4A-00</t>
         </is>
       </c>
       <c r="F26" s="8" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="8" t="n">
-        <v>13023</v>
+        <v>13024</v>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>A 4번 방 프리팹 (SILENT_Room_04_Structure, A·B 같은 방 껍데기)</t>
+          <t>A 5번 방 프리팹 (SILENT_Room_05_Structure, A·B 같은 방 껍데기)</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R04/SILENT_Room_04/Prefabs/SILENT_Room_04_Structure</t>
+          <t>Assets/2.Model/Prefabs/R05/SILENT_Room_05/Prefabs/SILENT_Room_05_Structure</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
@@ -1820,23 +1818,23 @@
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>R4A-00</t>
+          <t>R5A-00</t>
         </is>
       </c>
       <c r="F27" s="8" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="8" t="n">
-        <v>13024</v>
+        <v>13025</v>
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>A 5번 방 프리팹 (SILENT_Room_05_Structure, A·B 같은 방 껍데기)</t>
+          <t>A 6번 방 프리팹 (A·B 공통 구조 SILENT_Room_06_A_Structure)</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R05/SILENT_Room_05/Prefabs/SILENT_Room_05_Structure</t>
+          <t>Assets/2.Model/Prefabs/R06/SILENT_Room_06/Prefabs/SILENT_Room_06_A_Structure</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
@@ -1846,23 +1844,23 @@
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>R5A-00</t>
+          <t>R6A-00</t>
         </is>
       </c>
       <c r="F28" s="8" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="8" t="n">
-        <v>13025</v>
+        <v>13026</v>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>A 6번 방 프리팹 (A·B 공통 구조 SILENT_Room_06_A_Structure)</t>
+          <t>A 7번 방 프리팹 (A·B 공통 구조 R07_Structure, 천장 포함)</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R06/SILENT_Room_06/Prefabs/SILENT_Room_06_A_Structure</t>
+          <t>Assets/2.Model/Prefabs/R07/SILENT_Room_07/Prefabs/R07_Structure</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
@@ -1872,49 +1870,49 @@
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>R6A-00</t>
+          <t>R7A-00</t>
         </is>
       </c>
       <c r="F29" s="8" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="8" t="n">
-        <v>13026</v>
+        <v>13027</v>
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>A 7번 방 프리팹 (A·B 공통 구조 R07_Structure, 천장 포함)</t>
+          <t>B 1번 방 기본 프리팹 (A·B 공통: 맵 R01_Structure + 천장 Ceiling.007 + 문 막기 dver' + 앵커 R01_Points)</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R07/SILENT_Room_07/Prefabs/R07_Structure</t>
+          <t>Assets/2.Model/Prefabs/R01/SILENT_Room_01_Final/Prefabs/Room_01_Final</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>RoomA</t>
+          <t>RoomB</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
         <is>
-          <t>R7A-00</t>
+          <t>R1B-00</t>
         </is>
       </c>
       <c r="F30" s="8" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="8" t="n">
-        <v>13027</v>
+        <v>13028</v>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>B 1번 방 기본 프리팹 (A·B 공통: 맵 R01_Structure + 천장 Ceiling.007 + 문 막기 dver' + 앵커 R01_Points)</t>
+          <t>B 2번 방 프리팹 (천장 뺀 맵 R02_Structure + 앵커 R02_Points)</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R01/SILENT_Room_01_Final/Prefabs/Room_01_Final</t>
+          <t>Assets/2.Model/Prefabs/R02/SILENT_Room_02/Prefabs/SILENT_Room_02_Structure</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
@@ -1924,23 +1922,23 @@
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>R1B-00</t>
+          <t>R2B-00</t>
         </is>
       </c>
       <c r="F31" s="8" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="8" t="n">
-        <v>13028</v>
+        <v>13029</v>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>B 2번 방 프리팹 (천장 뺀 맵 R02_Structure + 앵커 R02_Points)</t>
+          <t>B 3번 방 프리팹 (SILENT_Room_03_Structure, A·B 같은 방 껍데기)</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R02/SILENT_Room_02/Prefabs/SILENT_Room_02_Structure</t>
+          <t>Assets/2.Model/Prefabs/R03/SILENT_Room_03/Prefabs/SILENT_Room_03_Structure</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
@@ -1950,23 +1948,23 @@
       </c>
       <c r="E32" s="8" t="inlineStr">
         <is>
-          <t>R2B-00</t>
+          <t>R3B-00</t>
         </is>
       </c>
       <c r="F32" s="8" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="8" t="n">
-        <v>13029</v>
+        <v>13030</v>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>B 3번 방 프리팹 (SILENT_Room_03_Structure, A·B 같은 방 껍데기)</t>
+          <t>B 4번 방 프리팹 (SILENT_Room_04_Structure, A·B 같은 방 껍데기)</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R03/SILENT_Room_03/Prefabs/SILENT_Room_03_Structure</t>
+          <t>Assets/2.Model/Prefabs/R04/SILENT_Room_04/Prefabs/SILENT_Room_04_Structure</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
@@ -1976,23 +1974,23 @@
       </c>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>R3B-00</t>
+          <t>R4B-00</t>
         </is>
       </c>
       <c r="F33" s="8" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="8" t="n">
-        <v>13030</v>
+        <v>13031</v>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>B 4번 방 프리팹 (SILENT_Room_04_Structure, A·B 같은 방 껍데기)</t>
+          <t>B 5번 방 프리팹 (SILENT_Room_05_Structure, A·B 같은 방 껍데기)</t>
         </is>
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R04/SILENT_Room_04/Prefabs/SILENT_Room_04_Structure</t>
+          <t>Assets/2.Model/Prefabs/R05/SILENT_Room_05/Prefabs/SILENT_Room_05_Structure</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
@@ -2002,23 +2000,23 @@
       </c>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t>R4B-00</t>
+          <t>R5B-00</t>
         </is>
       </c>
       <c r="F34" s="8" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="8" t="n">
-        <v>13031</v>
+        <v>13032</v>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>B 5번 방 프리팹 (SILENT_Room_05_Structure, A·B 같은 방 껍데기)</t>
+          <t>B 6번 방 프리팹 (A·B 공통 구조 SILENT_Room_06_A_Structure)</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R05/SILENT_Room_05/Prefabs/SILENT_Room_05_Structure</t>
+          <t>Assets/2.Model/Prefabs/R06/SILENT_Room_06/Prefabs/SILENT_Room_06_A_Structure</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
@@ -2028,23 +2026,23 @@
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>R5B-00</t>
+          <t>R6B-00</t>
         </is>
       </c>
       <c r="F35" s="8" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="8" t="n">
-        <v>13032</v>
+        <v>13033</v>
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>B 6번 방 프리팹 (A·B 공통 구조 SILENT_Room_06_A_Structure)</t>
+          <t>B 7번 방 프리팹 (A·B 공통 구조 R07_Structure, 천장 포함)</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R06/SILENT_Room_06/Prefabs/SILENT_Room_06_A_Structure</t>
+          <t>Assets/2.Model/Prefabs/R07/SILENT_Room_07/Prefabs/R07_Structure</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
@@ -2054,75 +2052,75 @@
       </c>
       <c r="E36" s="8" t="inlineStr">
         <is>
-          <t>R6B-00</t>
+          <t>R7B-00</t>
         </is>
       </c>
       <c r="F36" s="8" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="8" t="n">
-        <v>13033</v>
+        <v>13034</v>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>B 7번 방 프리팹 (A·B 공통 구조 R07_Structure, 천장 포함)</t>
+          <t>전선</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R07/SILENT_Room_07/Prefabs/R07_Structure</t>
+          <t>Prefabs/R4/Wire</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>RoomB</t>
+          <t>Room4</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
-          <t>R7B-00</t>
+          <t>R4B-01</t>
         </is>
       </c>
       <c r="F37" s="8" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="8" t="n">
-        <v>13034</v>
+        <v>13035</v>
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>전선</t>
+          <t>1번 방 기본 맵 (방 모델 전체)</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>Prefabs/R4/Wire</t>
+          <t>Assets/2.Model/Prefabs/Map/Room_01/Room_01</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
-          <t>Room4</t>
+          <t>Room1</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
-          <t>R4B-01</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F38" s="8" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="8" t="n">
-        <v>13035</v>
+        <v>13036</v>
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>1번 방 기본 맵 (방 모델 전체)</t>
+          <t>1번 방 문 (옛 것, 13002 공통 문으로 대체되어 안 씀)</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/Map/Room_01/Room_01</t>
+          <t>Assets/2.Model/Prefabs/R01/R01_Door</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
@@ -2135,20 +2133,24 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F39" s="8" t="n"/>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>14001|14005</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="n">
-        <v>13036</v>
+        <v>13037</v>
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>1번 방 문 (옛 것, 13002 공통 문으로 대체되어 안 씀)</t>
+          <t>1번 방 바닥 (방 모델 안 'Floor')</t>
         </is>
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R01/R01_Door</t>
+          <t>Assets/2.Model/Prefabs/Map/Room_01/Room_01</t>
         </is>
       </c>
       <c r="D40" s="8" t="inlineStr">
@@ -2161,19 +2163,15 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F40" s="8" t="inlineStr">
-        <is>
-          <t>14001|14005</t>
-        </is>
-      </c>
+      <c r="F40" s="8" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="8" t="n">
-        <v>13037</v>
+        <v>13038</v>
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>1번 방 바닥 (방 모델 안 'Floor')</t>
+          <t>1번 방 벽 1 (방 모델 안 'North wall')</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
@@ -2195,11 +2193,11 @@
     </row>
     <row r="42">
       <c r="A42" s="8" t="n">
-        <v>13038</v>
+        <v>13039</v>
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>1번 방 벽 1 (방 모델 안 'North wall')</t>
+          <t>1번 방 벽 2 (방 모델 안 'East wall north')</t>
         </is>
       </c>
       <c r="C42" s="8" t="inlineStr">
@@ -2221,11 +2219,11 @@
     </row>
     <row r="43">
       <c r="A43" s="8" t="n">
-        <v>13039</v>
+        <v>13040</v>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>1번 방 벽 2 (방 모델 안 'East wall north')</t>
+          <t>1번 방 벽 3 (방 모델 안 'South wall')</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
@@ -2247,11 +2245,11 @@
     </row>
     <row r="44">
       <c r="A44" s="8" t="n">
-        <v>13040</v>
+        <v>13041</v>
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>1번 방 벽 3 (방 모델 안 'South wall')</t>
+          <t>1번 방 벽 4 (방 모델 안 'West wall north')</t>
         </is>
       </c>
       <c r="C44" s="8" t="inlineStr">
@@ -2273,16 +2271,16 @@
     </row>
     <row r="45">
       <c r="A45" s="8" t="n">
-        <v>13041</v>
+        <v>13042</v>
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>1번 방 벽 4 (방 모델 안 'West wall north')</t>
+          <t>1번 방 바닥 카드 50장</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/Map/Room_01/Room_01</t>
+          <t>Assets/2.Model/Prefabs/R01/R01_FloorCard</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
@@ -2295,25 +2293,29 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F45" s="8" t="n"/>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>14007</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="n">
-        <v>13042</v>
+        <v>13043</v>
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>1번 방 바닥 카드 50장</t>
+          <t>글자 표시판 (LED, 1~6번 방 공용)</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R01/R01_FloorCard</t>
+          <t>Assets/2.Model/Prefabs/R01/R01_LEDPanel</t>
         </is>
       </c>
       <c r="D46" s="8" t="inlineStr">
         <is>
-          <t>Room1</t>
+          <t>Shared</t>
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr">
@@ -2323,22 +2325,22 @@
       </c>
       <c r="F46" s="8" t="inlineStr">
         <is>
-          <t>14007</t>
+          <t>14006</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="n">
-        <v>13043</v>
+        <v>13044</v>
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>1번 방 글자 표시판 (LED)</t>
+          <t>1번 방 가구 (수납장 2개)</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R01/R01_LEDPanel</t>
+          <t>Assets/2.Model/Prefabs/R01/R01_Furniture</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
@@ -2351,24 +2353,20 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F47" s="8" t="inlineStr">
-        <is>
-          <t>14006</t>
-        </is>
-      </c>
+      <c r="F47" s="8" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="8" t="n">
-        <v>13044</v>
+        <v>13045</v>
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>1번 방 가구 (수납장 2개)</t>
+          <t>1번 방 다이얼 테이블</t>
         </is>
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R01/R01_Furniture</t>
+          <t>Assets/2.Model/Prefabs/R01/R01_Dial_table</t>
         </is>
       </c>
       <c r="D48" s="8" t="inlineStr">
@@ -2385,16 +2383,16 @@
     </row>
     <row r="49">
       <c r="A49" s="8" t="n">
-        <v>13045</v>
+        <v>13046</v>
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>1번 방 다이얼 테이블</t>
+          <t>1번 방 다이얼 0</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R01/R01_Dial_table</t>
+          <t>Assets/2.Model/Prefabs/R01/PZ_R1_B_Dial_0</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
@@ -2407,20 +2405,24 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F49" s="8" t="n"/>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>14001|14002|14003</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="8" t="n">
-        <v>13046</v>
+        <v>13047</v>
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>1번 방 다이얼 0</t>
+          <t>1번 방 다이얼 1</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R01/PZ_R1_B_Dial_0</t>
+          <t>Assets/2.Model/Prefabs/R01/PZ_R1_B_Dial_1</t>
         </is>
       </c>
       <c r="D50" s="8" t="inlineStr">
@@ -2441,16 +2443,16 @@
     </row>
     <row r="51">
       <c r="A51" s="8" t="n">
-        <v>13047</v>
+        <v>13048</v>
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>1번 방 다이얼 1</t>
+          <t>1번 방 다이얼 2</t>
         </is>
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R01/PZ_R1_B_Dial_1</t>
+          <t>Assets/2.Model/Prefabs/R01/PZ_R1_B_Dial_2</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
@@ -2471,16 +2473,16 @@
     </row>
     <row r="52">
       <c r="A52" s="8" t="n">
-        <v>13048</v>
+        <v>13049</v>
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>1번 방 다이얼 2</t>
+          <t>1번 방 다이얼 3</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R01/PZ_R1_B_Dial_2</t>
+          <t>Assets/2.Model/Prefabs/R01/PZ_R1_B_Dial_3</t>
         </is>
       </c>
       <c r="D52" s="8" t="inlineStr">
@@ -2501,21 +2503,21 @@
     </row>
     <row r="53">
       <c r="A53" s="8" t="n">
-        <v>13049</v>
+        <v>13050</v>
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>1번 방 다이얼 3</t>
+          <t>2번 방 의자</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R01/PZ_R1_B_Dial_3</t>
+          <t>Assets/2.Model/Prefabs/R02/R02_A_Chair</t>
         </is>
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>Room1</t>
+          <t>Room2</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
@@ -2523,24 +2525,20 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F53" s="8" t="inlineStr">
-        <is>
-          <t>14001|14002|14003</t>
-        </is>
-      </c>
+      <c r="F53" s="8" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="8" t="n">
-        <v>13050</v>
+        <v>13051</v>
       </c>
       <c r="B54" s="8" t="inlineStr">
         <is>
-          <t>2번 방 의자</t>
+          <t>2번 방 조명</t>
         </is>
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R02/R02_A_Chair</t>
+          <t>Assets/2.Model/Prefabs/R02/R02_A_Light</t>
         </is>
       </c>
       <c r="D54" s="8" t="inlineStr">
@@ -2557,16 +2555,16 @@
     </row>
     <row r="55">
       <c r="A55" s="8" t="n">
-        <v>13051</v>
+        <v>13052</v>
       </c>
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>2번 방 조명</t>
+          <t>2번 방 테이블</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R02/R02_A_Light</t>
+          <t>Assets/2.Model/Prefabs/R02/R02_A_Table</t>
         </is>
       </c>
       <c r="D55" s="8" t="inlineStr">
@@ -2583,16 +2581,16 @@
     </row>
     <row r="56">
       <c r="A56" s="8" t="n">
-        <v>13052</v>
+        <v>13053</v>
       </c>
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>2번 방 테이블</t>
+          <t>2번 방 큰 풀 (A·B 공통)</t>
         </is>
       </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R02/R02_A_Table</t>
+          <t>Assets/2.Model/Prefabs/R02/R02_BigGrass</t>
         </is>
       </c>
       <c r="D56" s="8" t="inlineStr">
@@ -2609,16 +2607,16 @@
     </row>
     <row r="57">
       <c r="A57" s="8" t="n">
-        <v>13053</v>
+        <v>13054</v>
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>2번 방 큰 풀 (A·B 공통)</t>
+          <t>2번 방 작은 풀</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R02/R02_BigGrass</t>
+          <t>Assets/2.Model/Prefabs/R02/R02_B_SmallGrass</t>
         </is>
       </c>
       <c r="D57" s="8" t="inlineStr">
@@ -2635,16 +2633,16 @@
     </row>
     <row r="58">
       <c r="A58" s="8" t="n">
-        <v>13054</v>
+        <v>13055</v>
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>2번 방 작은 풀</t>
+          <t>2번 방 액자 Black</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R02/R02_B_SmallGrass</t>
+          <t>Assets/2.Model/Prefabs/R02/R02_B_BlackFrame</t>
         </is>
       </c>
       <c r="D58" s="8" t="inlineStr">
@@ -2661,16 +2659,16 @@
     </row>
     <row r="59">
       <c r="A59" s="8" t="n">
-        <v>13055</v>
+        <v>13056</v>
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>2번 방 액자 Black</t>
+          <t>2번 방 액자 Blue</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R02/R02_B_BlackFrame</t>
+          <t>Assets/2.Model/Prefabs/R02/R02_B_BlueFrame</t>
         </is>
       </c>
       <c r="D59" s="8" t="inlineStr">
@@ -2687,16 +2685,16 @@
     </row>
     <row r="60">
       <c r="A60" s="8" t="n">
-        <v>13056</v>
+        <v>13057</v>
       </c>
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t>2번 방 액자 Blue</t>
+          <t>2번 방 액자 Gray</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R02/R02_B_BlueFrame</t>
+          <t>Assets/2.Model/Prefabs/R02/R02_B_GrayFrame</t>
         </is>
       </c>
       <c r="D60" s="8" t="inlineStr">
@@ -2713,16 +2711,16 @@
     </row>
     <row r="61">
       <c r="A61" s="8" t="n">
-        <v>13057</v>
+        <v>13058</v>
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>2번 방 액자 Gray</t>
+          <t>2번 방 액자 Green</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R02/R02_B_GrayFrame</t>
+          <t>Assets/2.Model/Prefabs/R02/R02_B_GreenFrame</t>
         </is>
       </c>
       <c r="D61" s="8" t="inlineStr">
@@ -2739,16 +2737,16 @@
     </row>
     <row r="62">
       <c r="A62" s="8" t="n">
-        <v>13058</v>
+        <v>13059</v>
       </c>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>2번 방 액자 Green</t>
+          <t>2번 방 액자 Teal (Unity 이름 Mint)</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R02/R02_B_GreenFrame</t>
+          <t>Assets/2.Model/Prefabs/R02/R02_B_MintFrame</t>
         </is>
       </c>
       <c r="D62" s="8" t="inlineStr">
@@ -2765,16 +2763,16 @@
     </row>
     <row r="63">
       <c r="A63" s="8" t="n">
-        <v>13059</v>
+        <v>13060</v>
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>2번 방 액자 Teal (Unity 이름 Mint)</t>
+          <t>2번 방 액자 Navy</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R02/R02_B_MintFrame</t>
+          <t>Assets/2.Model/Prefabs/R02/R02_B_NavyFrame</t>
         </is>
       </c>
       <c r="D63" s="8" t="inlineStr">
@@ -2791,16 +2789,16 @@
     </row>
     <row r="64">
       <c r="A64" s="8" t="n">
-        <v>13060</v>
+        <v>13061</v>
       </c>
       <c r="B64" s="8" t="inlineStr">
         <is>
-          <t>2번 방 액자 Navy</t>
+          <t>2번 방 액자 Orange</t>
         </is>
       </c>
       <c r="C64" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R02/R02_B_NavyFrame</t>
+          <t>Assets/2.Model/Prefabs/R02/R02_B_OrangeFrame</t>
         </is>
       </c>
       <c r="D64" s="8" t="inlineStr">
@@ -2817,16 +2815,16 @@
     </row>
     <row r="65">
       <c r="A65" s="8" t="n">
-        <v>13061</v>
+        <v>13062</v>
       </c>
       <c r="B65" s="8" t="inlineStr">
         <is>
-          <t>2번 방 액자 Orange</t>
+          <t>2번 방 액자 Purple (Unity 이름 Pupple)</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R02/R02_B_OrangeFrame</t>
+          <t>Assets/2.Model/Prefabs/R02/R02_B_PuppleFrame</t>
         </is>
       </c>
       <c r="D65" s="8" t="inlineStr">
@@ -2843,16 +2841,16 @@
     </row>
     <row r="66">
       <c r="A66" s="8" t="n">
-        <v>13062</v>
+        <v>13063</v>
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>2번 방 액자 Purple (Unity 이름 Pupple)</t>
+          <t>2번 방 액자 Red</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R02/R02_B_PuppleFrame</t>
+          <t>Assets/2.Model/Prefabs/R02/R02_B_RedFrame</t>
         </is>
       </c>
       <c r="D66" s="8" t="inlineStr">
@@ -2869,16 +2867,16 @@
     </row>
     <row r="67">
       <c r="A67" s="8" t="n">
-        <v>13063</v>
+        <v>13064</v>
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>2번 방 액자 Red</t>
+          <t>2번 방 액자 Yellow</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R02/R02_B_RedFrame</t>
+          <t>Assets/2.Model/Prefabs/R02/R02_B_YellowFrame</t>
         </is>
       </c>
       <c r="D67" s="8" t="inlineStr">
@@ -2895,21 +2893,21 @@
     </row>
     <row r="68">
       <c r="A68" s="8" t="n">
-        <v>13064</v>
+        <v>13065</v>
       </c>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>2번 방 액자 Yellow</t>
+          <t>1번 방 바닥·벽·천장 묶음 (앵커 3개 포함)</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R02/R02_B_YellowFrame</t>
+          <t>Assets/2.Model/Prefabs/R01/R01_Serface</t>
         </is>
       </c>
       <c r="D68" s="8" t="inlineStr">
         <is>
-          <t>Room2</t>
+          <t>Room1</t>
         </is>
       </c>
       <c r="E68" s="8" t="inlineStr">
@@ -2921,16 +2919,16 @@
     </row>
     <row r="69">
       <c r="A69" s="8" t="n">
-        <v>13065</v>
+        <v>13066</v>
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>1번 방 바닥·벽·천장 묶음 (앵커 3개 포함)</t>
+          <t>1번 방 소품 묶음</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R01/R01_Serface</t>
+          <t>Assets/2.Model/Prefabs/R01/R01_Other</t>
         </is>
       </c>
       <c r="D69" s="8" t="inlineStr">
@@ -2947,16 +2945,16 @@
     </row>
     <row r="70">
       <c r="A70" s="8" t="n">
-        <v>13066</v>
+        <v>13067</v>
       </c>
       <c r="B70" s="8" t="inlineStr">
         <is>
-          <t>1번 방 소품 묶음</t>
+          <t>1번 방 바닥 카드 (A, SILENT_Room_01_Final의 Room_01_A_Cards)</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R01/R01_Other</t>
+          <t>Assets/2.Model/Prefabs/R01/R01_A_Cards</t>
         </is>
       </c>
       <c r="D70" s="8" t="inlineStr">
@@ -2969,20 +2967,24 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F70" s="8" t="n"/>
+      <c r="F70" s="8" t="inlineStr">
+        <is>
+          <t>14007</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="n">
-        <v>13067</v>
+        <v>13068</v>
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>1번 방 바닥 카드 (A, SILENT_Room_01_Final의 Room_01_A_Cards)</t>
+          <t>1번 방 천장 (SILENT_Room_01_Final의 Ceiling.007)</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R01/R01_A_Cards</t>
+          <t>Assets/2.Model/Prefabs/R01/R01_Ceiling</t>
         </is>
       </c>
       <c r="D71" s="8" t="inlineStr">
@@ -2995,24 +2997,20 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F71" s="8" t="inlineStr">
-        <is>
-          <t>14007</t>
-        </is>
-      </c>
+      <c r="F71" s="8" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="8" t="n">
-        <v>13068</v>
+        <v>13069</v>
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>1번 방 천장 (SILENT_Room_01_Final의 Ceiling.007)</t>
+          <t>1번 방 바닥·벽 단독 프리팹 (지금은 방 프리팹 Room_01_Final이 맵을 들고 있어 안 씀)</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R01/R01_Ceiling</t>
+          <t>Assets/2.Model/Prefabs/R01/R01_Structure</t>
         </is>
       </c>
       <c r="D72" s="8" t="inlineStr">
@@ -3029,16 +3027,16 @@
     </row>
     <row r="73">
       <c r="A73" s="8" t="n">
-        <v>13069</v>
+        <v>13070</v>
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>1번 방 바닥·벽 단독 프리팹 (지금은 방 프리팹 Room_01_Final이 맵을 들고 있어 안 씀)</t>
+          <t>1번 방 문 막기용 문 (SILENT_Room_01_Final의 dver', 열리지 않음)</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R01/R01_Structure</t>
+          <t>Assets/2.Model/Prefabs/R01/R01_Dver</t>
         </is>
       </c>
       <c r="D73" s="8" t="inlineStr">
@@ -3055,16 +3053,16 @@
     </row>
     <row r="74">
       <c r="A74" s="8" t="n">
-        <v>13070</v>
+        <v>13071</v>
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>1번 방 문 막기용 문 (SILENT_Room_01_Final의 dver', 열리지 않음)</t>
+          <t>1번 방 서랍장 (SILENT_Room_01_Final의 Hemnes.Drawer)</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R01/R01_Dver</t>
+          <t>Assets/2.Model/Prefabs/R01/R01_Drawer</t>
         </is>
       </c>
       <c r="D74" s="8" t="inlineStr">
@@ -3081,21 +3079,21 @@
     </row>
     <row r="75">
       <c r="A75" s="8" t="n">
-        <v>13071</v>
+        <v>13072</v>
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>1번 방 서랍장 (SILENT_Room_01_Final의 Hemnes.Drawer)</t>
+          <t>2번 방 천장 (SILENT_Room_02_Structure의 Ceiling.008)</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R01/R01_Drawer</t>
+          <t>Assets/2.Model/Prefabs/R02/R02_Ceiling</t>
         </is>
       </c>
       <c r="D75" s="8" t="inlineStr">
         <is>
-          <t>Room1</t>
+          <t>Room2</t>
         </is>
       </c>
       <c r="E75" s="8" t="inlineStr">
@@ -3107,16 +3105,16 @@
     </row>
     <row r="76">
       <c r="A76" s="8" t="n">
-        <v>13072</v>
+        <v>13073</v>
       </c>
       <c r="B76" s="8" t="inlineStr">
         <is>
-          <t>2번 방 천장 (SILENT_Room_02_Structure의 Ceiling.008)</t>
+          <t>2번 방 A 소품 묶음 (SILENT_Room_02_A_Objects)</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R02/R02_Ceiling</t>
+          <t>Assets/2.Model/Prefabs/R02/SILENT_Room_02/Prefabs/SILENT_Room_02_A_Objects</t>
         </is>
       </c>
       <c r="D76" s="8" t="inlineStr">
@@ -3133,16 +3131,16 @@
     </row>
     <row r="77">
       <c r="A77" s="8" t="n">
-        <v>13073</v>
+        <v>13074</v>
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>2번 방 A 소품 묶음 (SILENT_Room_02_A_Objects)</t>
+          <t>2번 방 B 소품 · 액자 묶음 (SILENT_Room_02_B_Objects)</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R02/SILENT_Room_02/Prefabs/SILENT_Room_02_A_Objects</t>
+          <t>Assets/2.Model/Prefabs/R02/SILENT_Room_02/Prefabs/SILENT_Room_02_B_Objects</t>
         </is>
       </c>
       <c r="D77" s="8" t="inlineStr">
@@ -3159,21 +3157,21 @@
     </row>
     <row r="78">
       <c r="A78" s="8" t="n">
-        <v>13074</v>
+        <v>13075</v>
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>2번 방 B 소품 · 액자 묶음 (SILENT_Room_02_B_Objects)</t>
+          <t>1번 방 A 전용 소품 묶음 (서랍장 Hemnes.Drawer + 바닥 카드 Room_01_A_Cards)</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R02/SILENT_Room_02/Prefabs/SILENT_Room_02_B_Objects</t>
+          <t>Assets/2.Model/Prefabs/R01/SILENT_Room_01_Final/Prefabs/Room_01_Final 1</t>
         </is>
       </c>
       <c r="D78" s="8" t="inlineStr">
         <is>
-          <t>Room2</t>
+          <t>Room1</t>
         </is>
       </c>
       <c r="E78" s="8" t="inlineStr">
@@ -3181,25 +3179,29 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F78" s="8" t="n"/>
+      <c r="F78" s="8" t="inlineStr">
+        <is>
+          <t>14007</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="n">
-        <v>13075</v>
+        <v>13076</v>
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>1번 방 A 전용 소품 묶음 (서랍장 Hemnes.Drawer + 바닥 카드 Room_01_A_Cards)</t>
+          <t>3번 방 천장 (SILENT_Room_03_Structure의 Ceiling.002)</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R01/SILENT_Room_01_Final/Prefabs/Room_01_Final 1</t>
+          <t>Assets/2.Model/Prefabs/R03/SILENT_Room_03/Prefabs/R03_Ceiling</t>
         </is>
       </c>
       <c r="D79" s="8" t="inlineStr">
         <is>
-          <t>Room1</t>
+          <t>Room3</t>
         </is>
       </c>
       <c r="E79" s="8" t="inlineStr">
@@ -3207,24 +3209,20 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F79" s="8" t="inlineStr">
-        <is>
-          <t>14007</t>
-        </is>
-      </c>
+      <c r="F79" s="8" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="8" t="n">
-        <v>13076</v>
+        <v>13077</v>
       </c>
       <c r="B80" s="8" t="inlineStr">
         <is>
-          <t>3번 방 천장 (SILENT_Room_03_Structure의 Ceiling.002)</t>
+          <t>3번 방 A 소품 묶음 (SILENT_Room_03_A_Objects)</t>
         </is>
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R03/SILENT_Room_03/Prefabs/R03_Ceiling</t>
+          <t>Assets/2.Model/Prefabs/R03/SILENT_Room_03/Prefabs/SILENT_Room_03_A_Objects</t>
         </is>
       </c>
       <c r="D80" s="8" t="inlineStr">
@@ -3241,16 +3239,16 @@
     </row>
     <row r="81">
       <c r="A81" s="8" t="n">
-        <v>13077</v>
+        <v>13078</v>
       </c>
       <c r="B81" s="8" t="inlineStr">
         <is>
-          <t>3번 방 A 소품 묶음 (SILENT_Room_03_A_Objects)</t>
+          <t>3번 방 B 소품 묶음 (SILENT_Room_03_B_Objects, 글자 표시판 PZ_R3_B_RewardDisplay 포함)</t>
         </is>
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R03/SILENT_Room_03/Prefabs/SILENT_Room_03_A_Objects</t>
+          <t>Assets/2.Model/Prefabs/R03/SILENT_Room_03/Prefabs/SILENT_Room_03_B_Objects</t>
         </is>
       </c>
       <c r="D81" s="8" t="inlineStr">
@@ -3267,21 +3265,21 @@
     </row>
     <row r="82">
       <c r="A82" s="8" t="n">
-        <v>13078</v>
+        <v>13079</v>
       </c>
       <c r="B82" s="8" t="inlineStr">
         <is>
-          <t>3번 방 B 소품 묶음 (SILENT_Room_03_B_Objects, 글자 표시판 PZ_R3_B_RewardDisplay 포함)</t>
+          <t>4번 방 천장 (SILENT_Room_04_Structure의 Ceiling.003)</t>
         </is>
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R03/SILENT_Room_03/Prefabs/SILENT_Room_03_B_Objects</t>
+          <t>Assets/2.Model/Prefabs/R04/SILENT_Room_04/Prefabs/R04_Ceiling</t>
         </is>
       </c>
       <c r="D82" s="8" t="inlineStr">
         <is>
-          <t>Room3</t>
+          <t>Room4</t>
         </is>
       </c>
       <c r="E82" s="8" t="inlineStr">
@@ -3293,16 +3291,16 @@
     </row>
     <row r="83">
       <c r="A83" s="8" t="n">
-        <v>13079</v>
+        <v>13080</v>
       </c>
       <c r="B83" s="8" t="inlineStr">
         <is>
-          <t>4번 방 천장 (SILENT_Room_04_Structure의 Ceiling.003)</t>
+          <t>4번 방 A 소품 묶음 (SILENT_Room_04_A_Objects, 메시 하나)</t>
         </is>
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R04/SILENT_Room_04/Prefabs/R04_Ceiling</t>
+          <t>Assets/2.Model/Prefabs/R04/SILENT_Room_04/Prefabs/SILENT_Room_04_A_Objects</t>
         </is>
       </c>
       <c r="D83" s="8" t="inlineStr">
@@ -3319,16 +3317,16 @@
     </row>
     <row r="84">
       <c r="A84" s="8" t="n">
-        <v>13080</v>
+        <v>13081</v>
       </c>
       <c r="B84" s="8" t="inlineStr">
         <is>
-          <t>4번 방 A 소품 묶음 (SILENT_Room_04_A_Objects, 메시 하나)</t>
+          <t>4번 방 B 소품 묶음 (SILENT_Room_04_B_Objects, 메시 하나)</t>
         </is>
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R04/SILENT_Room_04/Prefabs/SILENT_Room_04_A_Objects</t>
+          <t>Assets/2.Model/Prefabs/R04/SILENT_Room_04/Prefabs/SILENT_Room_04_B_Objects</t>
         </is>
       </c>
       <c r="D84" s="8" t="inlineStr">
@@ -3345,21 +3343,21 @@
     </row>
     <row r="85">
       <c r="A85" s="8" t="n">
-        <v>13081</v>
+        <v>13082</v>
       </c>
       <c r="B85" s="8" t="inlineStr">
         <is>
-          <t>4번 방 B 소품 묶음 (SILENT_Room_04_B_Objects, 메시 하나)</t>
+          <t>5번 방 천장 (SILENT_Room_05_Structure의 Ceiling.004)</t>
         </is>
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R04/SILENT_Room_04/Prefabs/SILENT_Room_04_B_Objects</t>
+          <t>Assets/2.Model/Prefabs/R05/SILENT_Room_05/Prefabs/R05_Ceiling</t>
         </is>
       </c>
       <c r="D85" s="8" t="inlineStr">
         <is>
-          <t>Room4</t>
+          <t>Room5</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr">
@@ -3371,16 +3369,16 @@
     </row>
     <row r="86">
       <c r="A86" s="8" t="n">
-        <v>13082</v>
+        <v>13083</v>
       </c>
       <c r="B86" s="8" t="inlineStr">
         <is>
-          <t>5번 방 천장 (SILENT_Room_05_Structure의 Ceiling.004)</t>
+          <t>5번 방 A 소품 묶음 (SILENT_Room_05_A_Objects, 공식판 · 종이 · 책상 포함)</t>
         </is>
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R05/SILENT_Room_05/Prefabs/R05_Ceiling</t>
+          <t>Assets/2.Model/Prefabs/R05/SILENT_Room_05/Prefabs/SILENT_Room_05_A_Objects</t>
         </is>
       </c>
       <c r="D86" s="8" t="inlineStr">
@@ -3397,16 +3395,16 @@
     </row>
     <row r="87">
       <c r="A87" s="8" t="n">
-        <v>13083</v>
+        <v>13084</v>
       </c>
       <c r="B87" s="8" t="inlineStr">
         <is>
-          <t>5번 방 A 소품 묶음 (SILENT_Room_05_A_Objects, 공식판 · 종이 · 책상 포함)</t>
+          <t>5번 방 B 소품 묶음 (SILENT_Room_05_B_Objects)</t>
         </is>
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R05/SILENT_Room_05/Prefabs/SILENT_Room_05_A_Objects</t>
+          <t>Assets/2.Model/Prefabs/R05/SILENT_Room_05/Prefabs/SILENT_Room_05_B_Objects</t>
         </is>
       </c>
       <c r="D87" s="8" t="inlineStr">
@@ -3423,21 +3421,21 @@
     </row>
     <row r="88">
       <c r="A88" s="8" t="n">
-        <v>13084</v>
+        <v>13085</v>
       </c>
       <c r="B88" s="8" t="inlineStr">
         <is>
-          <t>5번 방 B 소품 묶음 (SILENT_Room_05_B_Objects)</t>
+          <t>6번 방 천장 (SILENT_Room_06_A_Structure의 Ceiling.005)</t>
         </is>
       </c>
       <c r="C88" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R05/SILENT_Room_05/Prefabs/SILENT_Room_05_B_Objects</t>
+          <t>Assets/2.Model/Prefabs/R06/SILENT_Room_06/Prefabs/R06_Ceiling</t>
         </is>
       </c>
       <c r="D88" s="8" t="inlineStr">
         <is>
-          <t>Room5</t>
+          <t>Room6</t>
         </is>
       </c>
       <c r="E88" s="8" t="inlineStr">
@@ -3449,16 +3447,16 @@
     </row>
     <row r="89">
       <c r="A89" s="8" t="n">
-        <v>13085</v>
+        <v>13086</v>
       </c>
       <c r="B89" s="8" t="inlineStr">
         <is>
-          <t>6번 방 천장 (SILENT_Room_06_A_Structure의 Ceiling.005)</t>
+          <t>6번 방 A 소품 묶음 (SILENT_Room_06_A_Objects, 메시 하나)</t>
         </is>
       </c>
       <c r="C89" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R06/SILENT_Room_06/Prefabs/R06_Ceiling</t>
+          <t>Assets/2.Model/Prefabs/R06/SILENT_Room_06/Prefabs/SILENT_Room_06_A_Objects</t>
         </is>
       </c>
       <c r="D89" s="8" t="inlineStr">
@@ -3475,16 +3473,16 @@
     </row>
     <row r="90">
       <c r="A90" s="8" t="n">
-        <v>13086</v>
+        <v>13087</v>
       </c>
       <c r="B90" s="8" t="inlineStr">
         <is>
-          <t>6번 방 A 소품 묶음 (SILENT_Room_06_A_Objects, 메시 하나)</t>
+          <t>6번 방 B 소품 · TV 묶음 (SILENT_Room_06_B_Objects, 메시 하나 + TV 화면 자리 12개)</t>
         </is>
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R06/SILENT_Room_06/Prefabs/SILENT_Room_06_A_Objects</t>
+          <t>Assets/2.Model/Prefabs/R06/SILENT_Room_06/Prefabs/SILENT_Room_06_B_Objects</t>
         </is>
       </c>
       <c r="D90" s="8" t="inlineStr">
@@ -3501,21 +3499,21 @@
     </row>
     <row r="91">
       <c r="A91" s="8" t="n">
-        <v>13087</v>
+        <v>13088</v>
       </c>
       <c r="B91" s="8" t="inlineStr">
         <is>
-          <t>6번 방 B 소품 · TV 묶음 (SILENT_Room_06_B_Objects, 메시 하나 + TV 화면 자리 12개)</t>
+          <t>7번 방 소품 묶음 (SILENT_Room_07_Objects, 메시 하나)</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R06/SILENT_Room_06/Prefabs/SILENT_Room_06_B_Objects</t>
+          <t>Assets/2.Model/Prefabs/R07/SILENT_Room_07/Prefabs/SILENT_Room_07_Objects</t>
         </is>
       </c>
       <c r="D91" s="8" t="inlineStr">
         <is>
-          <t>Room6</t>
+          <t>Room7</t>
         </is>
       </c>
       <c r="E91" s="8" t="inlineStr">
@@ -3527,29 +3525,123 @@
     </row>
     <row r="92">
       <c r="A92" s="8" t="n">
-        <v>13088</v>
+        <v>13089</v>
       </c>
       <c r="B92" s="8" t="inlineStr">
         <is>
-          <t>7번 방 소품 묶음 (SILENT_Room_07_Objects, 메시 하나)</t>
+          <t>1번 방 4칸 다이얼 자물쇠 (Lock_1to9 모델)</t>
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R07/SILENT_Room_07/Prefabs/SILENT_Room_07_Objects</t>
+          <t>Assets/2.Model/Prefabs/R01/R01_Lock</t>
         </is>
       </c>
       <c r="D92" s="8" t="inlineStr">
         <is>
+          <t>Room1</t>
+        </is>
+      </c>
+      <c r="E92" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F92" s="8" t="inlineStr">
+        <is>
+          <t>14001|14002|14003</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="8" t="n">
+        <v>13090</v>
+      </c>
+      <c r="B93" s="8" t="inlineStr">
+        <is>
+          <t>5번 방 4칸 다이얼 자물쇠 (Padlock_4Dial_0to9 모델)</t>
+        </is>
+      </c>
+      <c r="C93" s="8" t="inlineStr">
+        <is>
+          <t>Assets/2.Model/Prefabs/R05/R05_Lock</t>
+        </is>
+      </c>
+      <c r="D93" s="8" t="inlineStr">
+        <is>
+          <t>Room5</t>
+        </is>
+      </c>
+      <c r="E93" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F93" s="8" t="inlineStr">
+        <is>
+          <t>14001|14002|14003</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="8" t="n">
+        <v>13091</v>
+      </c>
+      <c r="B94" s="8" t="inlineStr">
+        <is>
+          <t>6번 방 5칸 글자 다이얼 자물쇠 (Lock_06 모델)</t>
+        </is>
+      </c>
+      <c r="C94" s="8" t="inlineStr">
+        <is>
+          <t>Assets/2.Model/Prefabs/R06/R06_Lock</t>
+        </is>
+      </c>
+      <c r="D94" s="8" t="inlineStr">
+        <is>
+          <t>Room6</t>
+        </is>
+      </c>
+      <c r="E94" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F94" s="8" t="inlineStr">
+        <is>
+          <t>14001|14002|14003</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="8" t="n">
+        <v>13092</v>
+      </c>
+      <c r="B95" s="8" t="inlineStr">
+        <is>
+          <t>7번 방 B 6칸 색 다이얼 자물쇠 (안내 글자 SILENT, R07_Lock에서 안내 글자 순서만 바꿈)</t>
+        </is>
+      </c>
+      <c r="C95" s="8" t="inlineStr">
+        <is>
+          <t>Assets/2.Model/Prefabs/R07/R07B_Lock</t>
+        </is>
+      </c>
+      <c r="D95" s="8" t="inlineStr">
+        <is>
           <t>Room7</t>
         </is>
       </c>
-      <c r="E92" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F92" s="8" t="n"/>
+      <c r="E95" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F95" s="8" t="inlineStr">
+        <is>
+          <t>14001|14002|14003</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
LED PANEL 작업 완료
</commit_message>
<xml_diff>
--- a/EXCEL/SILENT_Asset_Datatable.xlsx
+++ b/EXCEL/SILENT_Asset_Datatable.xlsx
@@ -1118,7 +1118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="10" customWidth="1" style="10" min="1" max="1"/>
@@ -1795,7 +1795,7 @@
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>글자 표시판 (LED, 1~6번 방 공용)</t>
+          <t>1번 방 글자 표시판 (LED, 글자 L / Red)</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
@@ -1805,7 +1805,7 @@
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>Shared</t>
+          <t>Room1</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
@@ -1821,16 +1821,16 @@
     </row>
     <row r="29">
       <c r="A29" s="8" t="n">
-        <v>13072</v>
+        <v>13044</v>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>2번 방 천장 (SILENT_Room_02_Structure의 Ceiling.008)</t>
+          <t> 방 글자 표시판 (LED, 글자 I / Green)</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R02/R02_Ceiling</t>
+          <t>Assets/2.Model/Prefabs/R02/R02_LEDPanel</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
@@ -1843,25 +1843,29 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F29" s="8" t="n"/>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>14006</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="n">
-        <v>13073</v>
+        <v>13045</v>
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>2번 방 A 소품 묶음 (SILENT_Room_02_A_Objects)</t>
+          <t> 방 글자 표시판 (LED, 글자 S / Purple)</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R02/SILENT_Room_02/Prefabs/SILENT_Room_02_A_Objects</t>
+          <t>Assets/2.Model/Prefabs/R03/R03_LEDPanel</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>Room2</t>
+          <t>Room3</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
@@ -1869,25 +1873,29 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F30" s="8" t="n"/>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>14006</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="n">
-        <v>13074</v>
+        <v>13046</v>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>2번 방 B 소품 · 액자 묶음 (SILENT_Room_02_B_Objects)</t>
+          <t> 방 글자 표시판 (LED, 글자 T / Crimson)</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R02/SILENT_Room_02/Prefabs/SILENT_Room_02_B_Objects</t>
+          <t>Assets/2.Model/Prefabs/R04/R04_LEDPanel</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>Room2</t>
+          <t>Room4</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -1895,25 +1903,29 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F31" s="8" t="n"/>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>14006</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="n">
-        <v>13075</v>
+        <v>13047</v>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>1번 방 A 전용 소품 묶음 (서랍장 Hemnes.Drawer + 바닥 카드 Room_01_A_Cards)</t>
+          <t> 방 글자 표시판 (LED, 글자 E / Yellow)</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R01/SILENT_Room_01_Final/Prefabs/Room_01_Final 1</t>
+          <t>Assets/2.Model/Prefabs/R05/R05_LEDPanel</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>Room1</t>
+          <t>Room5</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
@@ -1923,27 +1935,27 @@
       </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
-          <t>14007</t>
+          <t>14006</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="n">
-        <v>13077</v>
+        <v>13048</v>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>3번 방 A 소품 묶음 (SILENT_Room_03_A_Objects)</t>
+          <t> 방 글자 표시판 (LED, 글자 N / Pink)</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R03/SILENT_Room_03/Prefabs/SILENT_Room_03_A_Objects</t>
+          <t>Assets/2.Model/Prefabs/R06/R06_LEDPanel</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>Room3</t>
+          <t>Room6</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
@@ -1951,25 +1963,29 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F33" s="8" t="n"/>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>14006</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="n">
-        <v>13078</v>
+        <v>13072</v>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>3번 방 B 소품 묶음 (SILENT_Room_03_B_Objects, 글자 표시판 PZ_R3_B_RewardDisplay 포함)</t>
+          <t>2번 방 천장 (SILENT_Room_02_Structure의 Ceiling.008)</t>
         </is>
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R03/SILENT_Room_03/Prefabs/SILENT_Room_03_B_Objects</t>
+          <t>Assets/2.Model/Prefabs/R02/R02_Ceiling</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>Room3</t>
+          <t>Room2</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
@@ -1981,21 +1997,21 @@
     </row>
     <row r="35">
       <c r="A35" s="8" t="n">
-        <v>13080</v>
+        <v>13073</v>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>4번 방 A 소품 묶음 (SILENT_Room_04_A_Objects, 메시 하나)</t>
+          <t>2번 방 A 소품 묶음 (SILENT_Room_02_A_Objects)</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R04/SILENT_Room_04/Prefabs/SILENT_Room_04_A_Objects</t>
+          <t>Assets/2.Model/Prefabs/R02/SILENT_Room_02/Prefabs/SILENT_Room_02_A_Objects</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>Room4</t>
+          <t>Room2</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
@@ -2007,21 +2023,21 @@
     </row>
     <row r="36">
       <c r="A36" s="8" t="n">
-        <v>13081</v>
+        <v>13074</v>
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>4번 방 B 소품 묶음 (SILENT_Room_04_B_Objects, 메시 하나)</t>
+          <t>2번 방 B 소품 · 액자 묶음 (SILENT_Room_02_B_Objects)</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R04/SILENT_Room_04/Prefabs/SILENT_Room_04_B_Objects</t>
+          <t>Assets/2.Model/Prefabs/R02/SILENT_Room_02/Prefabs/SILENT_Room_02_B_Objects</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>Room4</t>
+          <t>Room2</t>
         </is>
       </c>
       <c r="E36" s="8" t="inlineStr">
@@ -2033,21 +2049,21 @@
     </row>
     <row r="37">
       <c r="A37" s="8" t="n">
-        <v>13083</v>
+        <v>13075</v>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>5번 방 A 소품 묶음 (SILENT_Room_05_A_Objects, 공식판 · 종이 · 책상 포함)</t>
+          <t>1번 방 A 전용 소품 묶음 (서랍장 Hemnes.Drawer + 바닥 카드 Room_01_A_Cards)</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R05/SILENT_Room_05/Prefabs/SILENT_Room_05_A_Objects</t>
+          <t>Assets/2.Model/Prefabs/R01/SILENT_Room_01_Final/Prefabs/Room_01_Final 1</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>Room5</t>
+          <t>Room1</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
@@ -2055,25 +2071,29 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F37" s="8" t="n"/>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>14007</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="n">
-        <v>13084</v>
+        <v>13077</v>
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>5번 방 B 소품 묶음 (SILENT_Room_05_B_Objects)</t>
+          <t>3번 방 A 소품 묶음 (SILENT_Room_03_A_Objects)</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R05/SILENT_Room_05/Prefabs/SILENT_Room_05_B_Objects</t>
+          <t>Assets/2.Model/Prefabs/R03/SILENT_Room_03/Prefabs/SILENT_Room_03_A_Objects</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
-          <t>Room5</t>
+          <t>Room3</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
@@ -2085,21 +2105,21 @@
     </row>
     <row r="39">
       <c r="A39" s="8" t="n">
-        <v>13086</v>
+        <v>13078</v>
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>6번 방 A 소품 묶음 (SILENT_Room_06_A_Objects, 메시 하나)</t>
+          <t>3번 방 B 소품 묶음 (SILENT_Room_03_B_Objects, 글자 표시판 PZ_R3_B_RewardDisplay 포함)</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R06/SILENT_Room_06/Prefabs/SILENT_Room_06_A_Objects</t>
+          <t>Assets/2.Model/Prefabs/R03/SILENT_Room_03/Prefabs/SILENT_Room_03_B_Objects</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>Room6</t>
+          <t>Room3</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
@@ -2111,21 +2131,21 @@
     </row>
     <row r="40">
       <c r="A40" s="8" t="n">
-        <v>13087</v>
+        <v>13080</v>
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>6번 방 B 소품 · TV 묶음 (SILENT_Room_06_B_Objects, 메시 하나 + TV 화면 자리 12개)</t>
+          <t>4번 방 A 소품 묶음 (SILENT_Room_04_A_Objects, 메시 하나)</t>
         </is>
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R06/SILENT_Room_06/Prefabs/SILENT_Room_06_B_Objects</t>
+          <t>Assets/2.Model/Prefabs/R04/SILENT_Room_04/Prefabs/SILENT_Room_04_A_Objects</t>
         </is>
       </c>
       <c r="D40" s="8" t="inlineStr">
         <is>
-          <t>Room6</t>
+          <t>Room4</t>
         </is>
       </c>
       <c r="E40" s="8" t="inlineStr">
@@ -2137,21 +2157,21 @@
     </row>
     <row r="41">
       <c r="A41" s="8" t="n">
-        <v>13088</v>
+        <v>13081</v>
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>7번 방 소품 묶음 (SILENT_Room_07_Objects, 메시 하나)</t>
+          <t>4번 방 B 소품 묶음 (SILENT_Room_04_B_Objects, 메시 하나)</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R07/SILENT_Room_07/Prefabs/SILENT_Room_07_Objects</t>
+          <t>Assets/2.Model/Prefabs/R04/SILENT_Room_04/Prefabs/SILENT_Room_04_B_Objects</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>Room7</t>
+          <t>Room4</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
@@ -2163,21 +2183,21 @@
     </row>
     <row r="42">
       <c r="A42" s="8" t="n">
-        <v>13089</v>
+        <v>13083</v>
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>1번 방 4칸 다이얼 자물쇠 (Lock_1to9 모델)</t>
+          <t>5번 방 A 소품 묶음 (SILENT_Room_05_A_Objects, 공식판 · 종이 · 책상 포함)</t>
         </is>
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R01/R01_Lock</t>
+          <t>Assets/2.Model/Prefabs/R05/SILENT_Room_05/Prefabs/SILENT_Room_05_A_Objects</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr">
         <is>
-          <t>Room1</t>
+          <t>Room5</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr">
@@ -2185,24 +2205,20 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F42" s="8" t="inlineStr">
-        <is>
-          <t>14001|14002|14003</t>
-        </is>
-      </c>
+      <c r="F42" s="8" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="8" t="n">
-        <v>13090</v>
+        <v>13084</v>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>5번 방 4칸 다이얼 자물쇠 (Padlock_4Dial_0to9 모델)</t>
+          <t>5번 방 B 소품 묶음 (SILENT_Room_05_B_Objects)</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R05/R05_Lock</t>
+          <t>Assets/2.Model/Prefabs/R05/SILENT_Room_05/Prefabs/SILENT_Room_05_B_Objects</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
@@ -2215,24 +2231,20 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F43" s="8" t="inlineStr">
-        <is>
-          <t>14001|14002|14003</t>
-        </is>
-      </c>
+      <c r="F43" s="8" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="8" t="n">
-        <v>13091</v>
+        <v>13086</v>
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>6번 방 5칸 글자 다이얼 자물쇠 (Lock_06 모델)</t>
+          <t>6번 방 A 소품 묶음 (SILENT_Room_06_A_Objects, 메시 하나)</t>
         </is>
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R06/R06_Lock</t>
+          <t>Assets/2.Model/Prefabs/R06/SILENT_Room_06/Prefabs/SILENT_Room_06_A_Objects</t>
         </is>
       </c>
       <c r="D44" s="8" t="inlineStr">
@@ -2245,29 +2257,25 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F44" s="8" t="inlineStr">
-        <is>
-          <t>14001|14002|14003</t>
-        </is>
-      </c>
+      <c r="F44" s="8" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="8" t="n">
-        <v>13092</v>
+        <v>13087</v>
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>7번 방 B 6칸 색 다이얼 자물쇠 (안내 글자 SILENT, R07_Lock에서 안내 글자 순서만 바꿈)</t>
+          <t>6번 방 B 소품 · TV 묶음 (SILENT_Room_06_B_Objects, 메시 하나 + TV 화면 자리 12개)</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/R07/R07B_Lock</t>
+          <t>Assets/2.Model/Prefabs/R06/SILENT_Room_06/Prefabs/SILENT_Room_06_B_Objects</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>Room7</t>
+          <t>Room6</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
@@ -2275,29 +2283,25 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F45" s="8" t="inlineStr">
-        <is>
-          <t>14001|14002|14003</t>
-        </is>
-      </c>
+      <c r="F45" s="8" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="8" t="n">
-        <v>13093</v>
+        <v>13088</v>
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>플레이어 A 팔 + 무전기 (제스, 1인칭, v02 리그, 무전기는 RadioSocket.L)</t>
+          <t>7번 방 소품 묶음 (SILENT_Room_07_Objects, 메시 하나)</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Prefabs/Player/Arms_A_Model</t>
+          <t>Assets/2.Model/Prefabs/R07/SILENT_Room_07/Prefabs/SILENT_Room_07_Objects</t>
         </is>
       </c>
       <c r="D46" s="8" t="inlineStr">
         <is>
-          <t>Player</t>
+          <t>Room7</t>
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr">
@@ -2309,172 +2313,193 @@
     </row>
     <row r="47">
       <c r="A47" s="8" t="n">
+        <v>13089</v>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>1번 방 4칸 다이얼 자물쇠 (Lock_1to9 모델)</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>Assets/2.Model/Prefabs/R01/R01_Lock</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Room1</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>14001|14002|14003</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="n">
+        <v>13090</v>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>5번 방 4칸 다이얼 자물쇠 (Padlock_4Dial_0to9 모델)</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>Assets/2.Model/Prefabs/R05/R05_Lock</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Room5</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F48" s="8" t="inlineStr">
+        <is>
+          <t>14001|14002|14003</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="n">
+        <v>13091</v>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>6번 방 5칸 글자 다이얼 자물쇠 (Lock_06 모델)</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>Assets/2.Model/Prefabs/R06/R06_Lock</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Room6</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>14001|14002|14003</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="n">
+        <v>13092</v>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>7번 방 B 6칸 색 다이얼 자물쇠 (안내 글자 SILENT, R07_Lock에서 안내 글자 순서만 바꿈)</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>Assets/2.Model/Prefabs/R07/R07B_Lock</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Room7</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F50" s="8" t="inlineStr">
+        <is>
+          <t>14001|14002|14003</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="n">
+        <v>13093</v>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>플레이어 A 팔 + 무전기 (제스, 1인칭, v02 리그, 무전기는 RadioSocket.L)</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>Assets/2.Model/Prefabs/Player/Arms_A_Model</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F51" s="8" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="n">
         <v>13094</v>
       </c>
-      <c r="B47" s="8" t="inlineStr">
+      <c r="B52" s="8" t="inlineStr">
         <is>
           <t>플레이어 B 팔 + 무전기 (그로밋, 1인칭, v02 리그, 무전기는 RadioSocket.L)</t>
         </is>
       </c>
-      <c r="C47" s="8" t="inlineStr">
+      <c r="C52" s="8" t="inlineStr">
         <is>
           <t>Assets/2.Model/Prefabs/Player/Arms_B_Model</t>
         </is>
       </c>
-      <c r="D47" s="8" t="inlineStr">
+      <c r="D52" s="8" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F47" s="8" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>13100</v>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>1번방 라이트</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Assets/2.Model/Light/Room1_Light.prefab</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Room1</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>13101</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>2번방 라이트</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Assets/2.Model/Light/Room2_Light.prefab</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Room2</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="n">
-        <v>13102</v>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>3번방 라이트</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Assets/2.Model/Light/Room3_Light.prefab</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Room3</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="n">
-        <v>13103</v>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>4번방 라이트</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Assets/2.Model/Light/Room4_Light.prefab</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Room4</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
-        <v>13104</v>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>5번방 라이트</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Assets/2.Model/Light/Room5_Light.prefab</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Room5</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F52" s="8" t="n"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>13105</v>
+        <v>13100</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>6번방 라이트</t>
+          <t>1번방 라이트</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Assets/2.Model/Light/Room6_Light.prefab</t>
+          <t>Assets/2.Model/Light/Room1_Light.prefab</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Room6</t>
+          <t>Room1</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2485,24 +2510,149 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
+        <v>13101</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2번방 라이트</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Assets/2.Model/Light/Room2_Light.prefab</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Room2</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>13102</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>3번방 라이트</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Assets/2.Model/Light/Room3_Light.prefab</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Room3</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>13103</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>4번방 라이트</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Assets/2.Model/Light/Room4_Light.prefab</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Room4</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>13104</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>5번방 라이트</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Assets/2.Model/Light/Room5_Light.prefab</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Room5</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>13105</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>6번방 라이트</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Assets/2.Model/Light/Room6_Light.prefab</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Room6</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
         <v>13106</v>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>7번방 라이트</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>Assets/2.Model/Light/Room7_Light.prefab</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D59" t="inlineStr">
         <is>
           <t>Room7</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="E59" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>